<commit_message>
update more subjective results
</commit_message>
<xml_diff>
--- a/Eval/subjective/Thai Text-to-Speech (TTS) Listening Test (Responses).xlsx
+++ b/Eval/subjective/Thai Text-to-Speech (TTS) Listening Test (Responses).xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="86">
   <si>
     <t>Timestamp</t>
   </si>
@@ -291,6 +291,33 @@
   </si>
   <si>
     <t>ไอ้จ๋อมากินกล้วยเพลงโฟล์คซอง</t>
+  </si>
+  <si>
+    <t>ภาพนกกกกนกบนกรงนกตรงถนนสนธยา</t>
+  </si>
+  <si>
+    <t>ขอทราบอาการบด</t>
+  </si>
+  <si>
+    <t>ไอจ๋อมากินกล้วยเพลงโฟล์คซอง</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>นกกกกนกบนกรงนกตรงถนนสนธยา</t>
+  </si>
+  <si>
+    <t>อาการบด</t>
+  </si>
+  <si>
+    <t>ไอจ๋อนั่งกินกล้วยฟังโฟล์คซอง</t>
+  </si>
+  <si>
+    <t>[25–34]</t>
+  </si>
+  <si>
+    <t>ขอทราบอาการ</t>
   </si>
   <si>
     <t>Choose A1 or B1</t>
@@ -357,7 +384,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -372,6 +399,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -463,7 +496,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AA5" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AA8" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="27">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Title: Thai Speech Naturalness Evaluation_x000a_Description:_x000a_&quot;You will hear pairs of Thai speech samples synthesized from text containing challenging grapheme sequences. Please complete this test in a quiet environment using headphones. The task takes 12–15 minutes. Your responses will help understand Thai text-to-speech technology.&quot;_x000a_✅ I confirm I am a native Thai speaker with normal hearing_x000a_✅ I am using headphones in a quiet environment_x000a_(Disqualify respondents who skip these)_x000a_Test player_x000a__x000a_Do not forward or reuse the content!" id="2"/>
@@ -1144,6 +1177,252 @@
       </c>
       <c r="AA5" s="4"/>
     </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="5">
+        <v>46083.507540046296</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="U6" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="W6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="X6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA6" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="5">
+        <v>46083.514471689814</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="S7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="V7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="W7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="X7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA7" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="5">
+        <v>46083.55551663194</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="U8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="V8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="W8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="X8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z8" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">
@@ -1160,162 +1439,162 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="J1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>76</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="7" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="7" t="s">
         <v>66</v>
       </c>
     </row>

</xml_diff>